<commit_message>
Daily auto backup 2026-08-20 17:10
</commit_message>
<xml_diff>
--- a/check_new.xlsx
+++ b/check_new.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S9"/>
+  <dimension ref="A1:S15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -516,18 +516,18 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>3895762</t>
+          <t>6835016</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Story</t>
+          <t>Release</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Loganathan Murugan (MS/EIN32-VM)</t>
+          <t>Vinod Kumar Sengotuvelu (MS/EMB1-VM)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -540,12 +540,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>20-09-2023</t>
+          <t>27-03-2026</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>24-10-2023</t>
+          <t>No Date</t>
         </is>
       </c>
       <c r="I2" t="n">
@@ -585,18 +585,18 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>6835016</t>
+          <t>6955690</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Release</t>
+          <t>Defectfix</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Vinod Kumar Sengotuvelu (MS/EMB1-VM)</t>
+          <t>Balu Sreevaikundam Muthukrishnan (MS/EMB1-VM)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>27-03-2026</t>
+          <t>28-04-2026</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -654,18 +654,18 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>5718753</t>
+          <t>3895762</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Task</t>
+          <t>Story</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Anant R K Ashwin (MS/EHE2-VM)</t>
+          <t>Loganathan Murugan (MS/EIN32-VM)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -678,12 +678,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>13-05-2025</t>
+          <t>20-09-2023</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>26-02-2026</t>
+          <t>24-10-2023</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -717,24 +717,24 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>1003.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>6915158</t>
+          <t>7233844</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Defect</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Harini Rajagopal (MS/EIN6-SWC)</t>
+          <t>Priya Dharshini Arumugam (MS/EHE2-VM)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>20-04-2026</t>
+          <t>14-07-2026</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -774,16 +774,16 @@
         <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="P5" t="n">
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="R5" t="n">
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="S5" t="n">
         <v>0</v>
@@ -792,12 +792,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>6877077</t>
+          <t>7335702</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Story</t>
+          <t>Defect</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -816,19 +816,19 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>08-04-2026</t>
+          <t>10-08-2026</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>25-05-2026</t>
+          <t>17-08-2026</t>
         </is>
       </c>
       <c r="I6" t="n">
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
@@ -837,22 +837,22 @@
         <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="N6" t="n">
         <v>0</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P6" t="n">
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R6" t="n">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
@@ -861,18 +861,18 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>6771108</t>
+          <t>6021717</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Epic</t>
+          <t>Defect</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Anitha Anju (MS/EHE2-VM)</t>
+          <t>Swetha Sagili (MS/EBV3-SWC)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -885,19 +885,19 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>13-03-2026</t>
+          <t>07-08-2025</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>08-06-2026</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="I7" t="n">
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -906,22 +906,22 @@
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>0</v>
+        <v>2.5</v>
       </c>
       <c r="R7" t="n">
-        <v>25</v>
+        <v>2.5</v>
       </c>
       <c r="S7" t="n">
         <v>0</v>
@@ -930,18 +930,18 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>6124561</t>
+          <t>5911162</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Release</t>
+          <t>Defect</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Priya Dharshini Arumugam (MS/EHE2-VM)</t>
+          <t>Anirudhra C S (MS/EBD11-VM)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -954,114 +954,528 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>10-09-2025</t>
+          <t>07-07-2025</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>No Date</t>
+          <t>17-02-2026</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>248.75</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>628.1</v>
+        <v>0</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>354.25</v>
+        <v>20</v>
       </c>
       <c r="M8" t="n">
-        <v>628.1</v>
+        <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>105.5</v>
+        <v>20</v>
       </c>
       <c r="O8" t="n">
-        <v>724.25</v>
+        <v>0</v>
       </c>
       <c r="P8" t="n">
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>724.25</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>1352.35</v>
+        <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>6124561</t>
+          <t>5718753</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Release</t>
+          <t>Task</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
+          <t>Anant R K Ashwin (MS/EHE2-VM)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>26.71</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>13-05-2025</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>26-02-2026</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>6915158</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Harini Rajagopal (MS/EIN6-SWC)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>26.71</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>20-04-2026</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>No Date</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>6877077</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Story</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Anitha Anju (MS/EHE2-VM)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>26.71</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>08-04-2026</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>25-05-2026</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>25</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>25</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="n">
+        <v>25</v>
+      </c>
+      <c r="S11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>6771108</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Anitha Anju (MS/EHE2-VM)</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>26.71</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>13-03-2026</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>08-06-2026</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>25</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>25</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" t="n">
+        <v>25</v>
+      </c>
+      <c r="S12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>6970833</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Defectfix</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Amirthavarshini Ravi (MS/EMB1-VM)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>26.71</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>05-05-2026</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>21-05-2026</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>6124561</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Priya Dharshini Arumugam (MS/EHE2-VM)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>26.71</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>10-09-2025</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>No Date</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>248.75</v>
+      </c>
+      <c r="J14" t="n">
+        <v>628.1</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
+        <v>354.25</v>
+      </c>
+      <c r="M14" t="n">
+        <v>628.1</v>
+      </c>
+      <c r="N14" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="O14" t="n">
+        <v>707.75</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>707.75</v>
+      </c>
+      <c r="R14" t="n">
+        <v>1335.85</v>
+      </c>
+      <c r="S14" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>6124561</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Release</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
           <t>EXTERNAL Besson Lucas (TS, VM/ESB3)</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Germany</t>
         </is>
       </c>
-      <c r="F9" t="n">
+      <c r="F15" t="n">
         <v>93.48</v>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>10-09-2025</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>No Date</t>
         </is>
       </c>
-      <c r="I9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" t="n">
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
         <v>8</v>
       </c>
-      <c r="K9" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" t="n">
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
         <v>8</v>
       </c>
-      <c r="N9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0</v>
-      </c>
-      <c r="R9" t="n">
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" t="n">
         <v>8</v>
       </c>
-      <c r="S9" t="n">
+      <c r="S15" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>